<commit_message>
NHSNOnboarding: Fixed the HSLOC and organization codes, and added tabs in excel sheets for reference tables
</commit_message>
<xml_diff>
--- a/nhsn/NHSN-App-BFF/StaticAssets/excel-sheets/Cerner_Import_Sheet.xlsx
+++ b/nhsn/NHSN-App-BFF/StaticAssets/excel-sheets/Cerner_Import_Sheet.xlsx
@@ -1,14 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F057F7D-073A-43D5-8A29-6B440B2BC6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D51492D6-2948-4453-9D6A-104921B9250E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FHIR Import" sheetId="1" r:id="rId1"/>
+    <sheet name="HSLOC Reference" sheetId="2" r:id="rId2"/>
+    <sheet name="Encounter Reference" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="549">
   <si>
     <t>NHSN Link - FHIR Server &amp; Patients of Interest Import Sheet</t>
   </si>
@@ -147,63 +149,63 @@
     <t>Census Acquisition Frequency - Hours</t>
   </si>
   <si>
+    <t>Yes - if Minutes not provided</t>
+  </si>
+  <si>
+    <t>This setting determines the frequency in which NHSNLink will attempt to get the latest census results.</t>
+  </si>
+  <si>
+    <t>censusFreqMinutes</t>
+  </si>
+  <si>
+    <t>Census Acquisition Frequency - Minutes</t>
+  </si>
+  <si>
+    <t>Yes - if Hours not provided; must be ≥5 min if Hours is blank</t>
+  </si>
+  <si>
+    <t>sftpHost</t>
+  </si>
+  <si>
+    <t>SFTP Host URL</t>
+  </si>
+  <si>
+    <t>The hostname or IP address of your facility's SFTP server that NHSNLink will connect to for file exchange.</t>
+  </si>
+  <si>
+    <t>sftpPort</t>
+  </si>
+  <si>
+    <t>SFTP Host URL Port</t>
+  </si>
+  <si>
+    <t>The port number used to connect to your facility's SFTP server (commonly 22 for SFTP).</t>
+  </si>
+  <si>
+    <t>sftpUsername</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Optional. Only needed if your facility's SFTP server requires basic authentication.</t>
+  </si>
+  <si>
+    <t>sftpPassword</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>remoteDirectory</t>
+  </si>
+  <si>
+    <t>Remote Directory</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Yes - if Minutes not provided</t>
-  </si>
-  <si>
-    <t>This setting determines the frequency in which NHSNLink will attempt to get the latest census results.</t>
-  </si>
-  <si>
-    <t>censusFreqMinutes</t>
-  </si>
-  <si>
-    <t>Census Acquisition Frequency - Minutes</t>
-  </si>
-  <si>
-    <t>Yes - if Hours not provided; must be ≥5 min if Hours is blank</t>
-  </si>
-  <si>
-    <t>sftpHost</t>
-  </si>
-  <si>
-    <t>SFTP Host URL</t>
-  </si>
-  <si>
-    <t>The hostname or IP address of your facility's SFTP server that NHSNLink will connect to for file exchange.</t>
-  </si>
-  <si>
-    <t>sftpPort</t>
-  </si>
-  <si>
-    <t>SFTP Host URL Port</t>
-  </si>
-  <si>
-    <t>The port number used to connect to your facility's SFTP server (commonly 22 for SFTP).</t>
-  </si>
-  <si>
-    <t>sftpUsername</t>
-  </si>
-  <si>
-    <t>Username</t>
-  </si>
-  <si>
-    <t>Optional. Only needed if your facility's SFTP server requires basic authentication.</t>
-  </si>
-  <si>
-    <t>sftpPassword</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>remoteDirectory</t>
-  </si>
-  <si>
-    <t>Remote Directory</t>
-  </si>
-  <si>
     <t>removeFilesAfterProcessing</t>
   </si>
   <si>
@@ -237,10 +239,10 @@
     <t>Organization Identification — Location Types</t>
   </si>
   <si>
-    <t>Location Type Code</t>
-  </si>
-  <si>
-    <t>Location Alias</t>
+    <t>Location.type.code</t>
+  </si>
+  <si>
+    <t>Location.alias</t>
   </si>
   <si>
     <t>Maps FHIR Location Type code(s) to an alias used to identify locations belonging to your facility.</t>
@@ -261,9 +263,6 @@
     <t>Your (local) Code</t>
   </si>
   <si>
-    <t>Location.alias.value</t>
-  </si>
-  <si>
     <t>HSLOC Code</t>
   </si>
   <si>
@@ -276,6 +275,9 @@
     <t>Encounter Mapping</t>
   </si>
   <si>
+    <t>Required - (At least one Encounter.type Code System is required. If Local Encounter.type Code, Reference Code System, or Reference Code is entered, all three must be entered)</t>
+  </si>
+  <si>
     <t>Encounter.type Code System</t>
   </si>
   <si>
@@ -289,13 +291,1402 @@
   </si>
   <si>
     <t>Maps your local Encounter.type codes to their standard reference code system and code.</t>
+  </si>
+  <si>
+    <t>1110-6</t>
+  </si>
+  <si>
+    <t>Allergy Clinic</t>
+  </si>
+  <si>
+    <t>1133-8</t>
+  </si>
+  <si>
+    <t>Pediatric Orthopedic Clinic</t>
+  </si>
+  <si>
+    <t>1046-2</t>
+  </si>
+  <si>
+    <t>Pediatric Neurosurgical Critical Care</t>
+  </si>
+  <si>
+    <t>1126-2</t>
+  </si>
+  <si>
+    <t>Ear, Nose, Throat Clinic</t>
+  </si>
+  <si>
+    <t>1018-1</t>
+  </si>
+  <si>
+    <t>Infusion Center</t>
+  </si>
+  <si>
+    <t>1127-0</t>
+  </si>
+  <si>
+    <t>Pain Clinic</t>
+  </si>
+  <si>
+    <t>1221-1</t>
+  </si>
+  <si>
+    <t>Long Term Acute Care Ward</t>
+  </si>
+  <si>
+    <t>1058-7</t>
+  </si>
+  <si>
+    <t>Labor and Delivery Ward</t>
+  </si>
+  <si>
+    <t>1164-3</t>
+  </si>
+  <si>
+    <t>Ventilator Dependent Unit</t>
+  </si>
+  <si>
+    <t>1061-1</t>
+  </si>
+  <si>
+    <t>Medical-Surgical Ward</t>
+  </si>
+  <si>
+    <t>1044-7</t>
+  </si>
+  <si>
+    <t>Pediatric Medical Critical Care</t>
+  </si>
+  <si>
+    <t>1116-3</t>
+  </si>
+  <si>
+    <t>Diabetes-Endocrinology Clinic</t>
+  </si>
+  <si>
+    <t>1165-0</t>
+  </si>
+  <si>
+    <t>Inpatient Hospice</t>
+  </si>
+  <si>
+    <t>1081-9</t>
+  </si>
+  <si>
+    <t>Pediatric Medical-Surgical Ward</t>
+  </si>
+  <si>
+    <t>1066-0</t>
+  </si>
+  <si>
+    <t>Orthopedic Trauma Ward</t>
+  </si>
+  <si>
+    <t>1189-0</t>
+  </si>
+  <si>
+    <t>Morgue/Autopsy Room</t>
+  </si>
+  <si>
+    <t>1139-5</t>
+  </si>
+  <si>
+    <t>Well Baby Clinic</t>
+  </si>
+  <si>
+    <t>1195-7</t>
+  </si>
+  <si>
+    <t>Blood Collection (Blood Drive Campaign)</t>
+  </si>
+  <si>
+    <t>1194-0</t>
+  </si>
+  <si>
+    <t>Home-based Hospice</t>
+  </si>
+  <si>
+    <t>1245-0</t>
+  </si>
+  <si>
+    <t>Ambulatory Surgery Recovery Room</t>
+  </si>
+  <si>
+    <t>1227-8</t>
+  </si>
+  <si>
+    <t>Oncology Step Down Unit</t>
+  </si>
+  <si>
+    <t>1190-8</t>
+  </si>
+  <si>
+    <t>Soiled Utility Area</t>
+  </si>
+  <si>
+    <t>1040-5</t>
+  </si>
+  <si>
+    <t>Neonatal Critical Care (Level III)</t>
+  </si>
+  <si>
+    <t>1178-3</t>
+  </si>
+  <si>
+    <t>Transport Service</t>
+  </si>
+  <si>
+    <t>1038-9</t>
+  </si>
+  <si>
+    <t>Well Newborn Nursery (Level I)</t>
+  </si>
+  <si>
+    <t>1122-1</t>
+  </si>
+  <si>
+    <t>Genetics Clinic</t>
+  </si>
+  <si>
+    <t>1220-3</t>
+  </si>
+  <si>
+    <t>Long Term Acute Care Intensive Care Unit</t>
+  </si>
+  <si>
+    <t>1246-8</t>
+  </si>
+  <si>
+    <t>Outpatient Ambulatory Pediatric Surgery Center</t>
+  </si>
+  <si>
+    <t>1007-4</t>
+  </si>
+  <si>
+    <t>Endoscopy Suite</t>
+  </si>
+  <si>
+    <t>1008-2</t>
+  </si>
+  <si>
+    <t>Radiology</t>
+  </si>
+  <si>
+    <t>1141-1</t>
+  </si>
+  <si>
+    <t>Physician's Office</t>
+  </si>
+  <si>
+    <t>1214-6</t>
+  </si>
+  <si>
+    <t>Long Term Acute Care Pediatric Ward</t>
+  </si>
+  <si>
+    <t>1125-4</t>
+  </si>
+  <si>
+    <t>Orthopedic Clinic</t>
+  </si>
+  <si>
+    <t>1147-8</t>
+  </si>
+  <si>
+    <t>Blood Collection Center</t>
+  </si>
+  <si>
+    <t>1009-0</t>
+  </si>
+  <si>
+    <t>Pulmonary Function Testing</t>
+  </si>
+  <si>
+    <t>1182-5</t>
+  </si>
+  <si>
+    <t>Housekeeping/Environmental Services</t>
+  </si>
+  <si>
+    <t>1117-1</t>
+  </si>
+  <si>
+    <t>Family Medicine Clinic</t>
+  </si>
+  <si>
+    <t>1156-9</t>
+  </si>
+  <si>
+    <t>Prenatal Clinic</t>
+  </si>
+  <si>
+    <t>1161-9</t>
+  </si>
+  <si>
+    <t>Holistic Medicine Center</t>
+  </si>
+  <si>
+    <t>1029-8</t>
+  </si>
+  <si>
+    <t>Medical-Surgical Critical Care</t>
+  </si>
+  <si>
+    <t>1103-1</t>
+  </si>
+  <si>
+    <t>Chronic Alzheimer's Unit</t>
+  </si>
+  <si>
+    <t>1065-2</t>
+  </si>
+  <si>
+    <t>Orthopedic Ward</t>
+  </si>
+  <si>
+    <t>1250-0</t>
+  </si>
+  <si>
+    <t>Facility-wide Inpatient (FacWIDEIn)</t>
+  </si>
+  <si>
+    <t>1033-0</t>
+  </si>
+  <si>
+    <t>Respiratory Critical Care</t>
+  </si>
+  <si>
+    <t>1138-7</t>
+  </si>
+  <si>
+    <t>Pediatric Rheumatology Clinic</t>
+  </si>
+  <si>
+    <t>1134-6</t>
+  </si>
+  <si>
+    <t>Pediatric Scoliosis Clinic</t>
+  </si>
+  <si>
+    <t>1025-6</t>
+  </si>
+  <si>
+    <t>Trauma Critical Care</t>
+  </si>
+  <si>
+    <t>1272-4</t>
+  </si>
+  <si>
+    <t>Onsite Overflow Critical Care</t>
+  </si>
+  <si>
+    <t>1159-3</t>
+  </si>
+  <si>
+    <t>Wound Ostomy Continence Clinic</t>
+  </si>
+  <si>
+    <t>1011-6</t>
+  </si>
+  <si>
+    <t>Clinical Chemistry Laboratory</t>
+  </si>
+  <si>
+    <t>1179-1</t>
+  </si>
+  <si>
+    <t>Pharmacy</t>
+  </si>
+  <si>
+    <t>1118-9</t>
+  </si>
+  <si>
+    <t>Gastrointestinal Clinic</t>
+  </si>
+  <si>
+    <t>1019-9</t>
+  </si>
+  <si>
+    <t>Specimen Collection Area (Healthcare)</t>
+  </si>
+  <si>
+    <t>1078-5</t>
+  </si>
+  <si>
+    <t>Pediatric Burn Ward</t>
+  </si>
+  <si>
+    <t>1145-2</t>
+  </si>
+  <si>
+    <t>Behavioral Health Clinic</t>
+  </si>
+  <si>
+    <t>1258-3</t>
+  </si>
+  <si>
+    <t>Long Term Care Facility General Nursing Unit</t>
+  </si>
+  <si>
+    <t>1172-6</t>
+  </si>
+  <si>
+    <t>School Infirmary</t>
+  </si>
+  <si>
+    <t>1039-7</t>
+  </si>
+  <si>
+    <t>Neonatal Critical Care (Level II/III)</t>
+  </si>
+  <si>
+    <t>1082-7</t>
+  </si>
+  <si>
+    <t>Pediatric Neurology Ward</t>
+  </si>
+  <si>
+    <t>1055-3</t>
+  </si>
+  <si>
+    <t>Genitourinary Ward</t>
+  </si>
+  <si>
+    <t>1219-5</t>
+  </si>
+  <si>
+    <t>Outpatient Hemodialysis Clinic (in Inpatient Facility)</t>
+  </si>
+  <si>
+    <t>1150-2</t>
+  </si>
+  <si>
+    <t>Dental Clinic</t>
+  </si>
+  <si>
+    <t>1102-3</t>
+  </si>
+  <si>
+    <t>Chronic Care Unit</t>
+  </si>
+  <si>
+    <t>1171-8</t>
+  </si>
+  <si>
+    <t>Jail Unit</t>
+  </si>
+  <si>
+    <t>1207-0</t>
+  </si>
+  <si>
+    <t>Therapeutic Apheresis Clinic</t>
+  </si>
+  <si>
+    <t>1054-6</t>
+  </si>
+  <si>
+    <t>Gastrointestinal Ward</t>
+  </si>
+  <si>
+    <t>1016-5</t>
+  </si>
+  <si>
+    <t>Virology Laboratory</t>
+  </si>
+  <si>
+    <t>1059-5</t>
+  </si>
+  <si>
+    <t>Labor, Delivery, Recovery, Postpartum Suite</t>
+  </si>
+  <si>
+    <t>1091-8</t>
+  </si>
+  <si>
+    <t>Pediatric Dialysis Specialty Care Area</t>
+  </si>
+  <si>
+    <t>1095-9</t>
+  </si>
+  <si>
+    <t>Cesarean Section Room/Suite</t>
+  </si>
+  <si>
+    <t>1203-9</t>
+  </si>
+  <si>
+    <t>Interventional Radiology</t>
+  </si>
+  <si>
+    <t>1222-9</t>
+  </si>
+  <si>
+    <t>Long Term Acute Care Pediatric Intensive Care Unit</t>
+  </si>
+  <si>
+    <t>1187-4</t>
+  </si>
+  <si>
+    <t>Central Trash Area</t>
+  </si>
+  <si>
+    <t>1185-8</t>
+  </si>
+  <si>
+    <t>Blood Bank</t>
+  </si>
+  <si>
+    <t>1210-4</t>
+  </si>
+  <si>
+    <t>Adult Mixed Acuity Unit</t>
+  </si>
+  <si>
+    <t>1108-0</t>
+  </si>
+  <si>
+    <t>Emergency Department</t>
+  </si>
+  <si>
+    <t>1104-9</t>
+  </si>
+  <si>
+    <t>Chronic Behavioral Health/Psych Unit</t>
+  </si>
+  <si>
+    <t>1249-2</t>
+  </si>
+  <si>
+    <t>Pediatric Outpatient Operating Room/Suite (Detached)</t>
+  </si>
+  <si>
+    <t>1115-5</t>
+  </si>
+  <si>
+    <t>Dermatology Clinic</t>
+  </si>
+  <si>
+    <t>1268-2</t>
+  </si>
+  <si>
+    <t>Outpatient Hemodialysis Clinic - Acute Kidney Injury</t>
+  </si>
+  <si>
+    <t>1042-1</t>
+  </si>
+  <si>
+    <t>Pediatric Burn Critical Care</t>
+  </si>
+  <si>
+    <t>1255-9</t>
+  </si>
+  <si>
+    <t>Long Term Care Facility Dementia Unit</t>
+  </si>
+  <si>
+    <t>1067-8</t>
+  </si>
+  <si>
+    <t>Plastic Surgery Ward</t>
+  </si>
+  <si>
+    <t>1077-7</t>
+  </si>
+  <si>
+    <t>Pediatric Behavioral Health Ward</t>
+  </si>
+  <si>
+    <t>1261-7</t>
+  </si>
+  <si>
+    <t>Centralized Transfusion Service</t>
+  </si>
+  <si>
+    <t>1243-5</t>
+  </si>
+  <si>
+    <t>Ambulatory Surgery Center</t>
+  </si>
+  <si>
+    <t>1205-4</t>
+  </si>
+  <si>
+    <t>Antenatal Care Ward</t>
+  </si>
+  <si>
+    <t>1105-6</t>
+  </si>
+  <si>
+    <t>Chronic Rehabilitation Unit</t>
+  </si>
+  <si>
+    <t>1142-9</t>
+  </si>
+  <si>
+    <t>Rheumatology Clinic</t>
+  </si>
+  <si>
+    <t>1160-1</t>
+  </si>
+  <si>
+    <t>Urgent Care Center</t>
+  </si>
+  <si>
+    <t>1085-0</t>
+  </si>
+  <si>
+    <t>Pediatric Rehabilitation Ward (within Hospital)</t>
+  </si>
+  <si>
+    <t>1051-2</t>
+  </si>
+  <si>
+    <t>Behavioral Health/Psych Ward</t>
+  </si>
+  <si>
+    <t>1086-8</t>
+  </si>
+  <si>
+    <t>Pediatric Surgical Ward</t>
+  </si>
+  <si>
+    <t>1032-2</t>
+  </si>
+  <si>
+    <t>Surgical Cardiothoracic Critical Care</t>
+  </si>
+  <si>
+    <t>1017-3</t>
+  </si>
+  <si>
+    <t>Hyperbaric Oxygen Center</t>
+  </si>
+  <si>
+    <t>1069-4</t>
+  </si>
+  <si>
+    <t>Pulmonary Ward</t>
+  </si>
+  <si>
+    <t>1079-3</t>
+  </si>
+  <si>
+    <t>Pediatric Ear, Nose, Throat Ward</t>
+  </si>
+  <si>
+    <t>1128-8</t>
+  </si>
+  <si>
+    <t>Pediatric Clinic</t>
+  </si>
+  <si>
+    <t>1035-5</t>
+  </si>
+  <si>
+    <t>Neurologic Critical Care</t>
+  </si>
+  <si>
+    <t>1212-0</t>
+  </si>
+  <si>
+    <t>Mixed Age Mixed Acuity Unit</t>
+  </si>
+  <si>
+    <t>1198-1</t>
+  </si>
+  <si>
+    <t>Dialysis Specialty Care Area</t>
+  </si>
+  <si>
+    <t>1132-0</t>
+  </si>
+  <si>
+    <t>Pediatric Diabetes-Endocrinology Clinic</t>
+  </si>
+  <si>
+    <t>1175-9</t>
+  </si>
+  <si>
+    <t>Mobile MRI/CT</t>
+  </si>
+  <si>
+    <t>1080-1</t>
+  </si>
+  <si>
+    <t>Pediatric Genitourinary Ward</t>
+  </si>
+  <si>
+    <t>1075-1</t>
+  </si>
+  <si>
+    <t>Adolescent Behavioral Health Ward</t>
+  </si>
+  <si>
+    <t>1062-9</t>
+  </si>
+  <si>
+    <t>Neurology Ward</t>
+  </si>
+  <si>
+    <t>1129-6</t>
+  </si>
+  <si>
+    <t>Pediatric Cardiology Center</t>
+  </si>
+  <si>
+    <t>1256-7</t>
+  </si>
+  <si>
+    <t>Long Term Care Facility Psychiatric Unit</t>
+  </si>
+  <si>
+    <t>1031-4</t>
+  </si>
+  <si>
+    <t>Neurosurgical Critical Care</t>
+  </si>
+  <si>
+    <t>1247-6</t>
+  </si>
+  <si>
+    <t>Outpatient Ambulatory Plastic Surgery Center</t>
+  </si>
+  <si>
+    <t>1131-2</t>
+  </si>
+  <si>
+    <t>Pediatric Dermatology Clinic</t>
+  </si>
+  <si>
+    <t>1196-5</t>
+  </si>
+  <si>
+    <t>Specimen Collection Area (Community)</t>
+  </si>
+  <si>
+    <t>1223-7</t>
+  </si>
+  <si>
+    <t>Oncology Medical Critical Care</t>
+  </si>
+  <si>
+    <t>1259-1</t>
+  </si>
+  <si>
+    <t>Long Term Care Facility Ventilator Dependent Unit</t>
+  </si>
+  <si>
+    <t>1026-4</t>
+  </si>
+  <si>
+    <t>Burn Critical Care</t>
+  </si>
+  <si>
+    <t>1169-2</t>
+  </si>
+  <si>
+    <t>Post-Anesthesia Care Unit</t>
+  </si>
+  <si>
+    <t>1005-8</t>
+  </si>
+  <si>
+    <t>Cardiac Catheterization Room/Suite</t>
+  </si>
+  <si>
+    <t>1204-7</t>
+  </si>
+  <si>
+    <t>Location outside facility</t>
+  </si>
+  <si>
+    <t>1113-0</t>
+  </si>
+  <si>
+    <t>Cardiology Clinic</t>
+  </si>
+  <si>
+    <t>1096-7</t>
+  </si>
+  <si>
+    <t>Operating Room/Suite</t>
+  </si>
+  <si>
+    <t>1071-0</t>
+  </si>
+  <si>
+    <t>Stroke (Acute) Ward</t>
+  </si>
+  <si>
+    <t>1192-4</t>
+  </si>
+  <si>
+    <t>Home Care</t>
+  </si>
+  <si>
+    <t>1183-3</t>
+  </si>
+  <si>
+    <t>Laundry Room</t>
+  </si>
+  <si>
+    <t>1045-4</t>
+  </si>
+  <si>
+    <t>Pediatric Medical-Surgical Critical Care</t>
+  </si>
+  <si>
+    <t>1154-4</t>
+  </si>
+  <si>
+    <t>HIV Clinic</t>
+  </si>
+  <si>
+    <t>1151-0</t>
+  </si>
+  <si>
+    <t>Occupational Health Clinic</t>
+  </si>
+  <si>
+    <t>1248-4</t>
+  </si>
+  <si>
+    <t>Pediatric Outpatient Operating Room/Suite (Attached)</t>
+  </si>
+  <si>
+    <t>1083-5</t>
+  </si>
+  <si>
+    <t>Pediatric Neurosurgical Ward</t>
+  </si>
+  <si>
+    <t>1263-3</t>
+  </si>
+  <si>
+    <t>Non-CMS Hospital Units</t>
+  </si>
+  <si>
+    <t>1226-0</t>
+  </si>
+  <si>
+    <t>Oncology Leukemia Ward</t>
+  </si>
+  <si>
+    <t>1233-6</t>
+  </si>
+  <si>
+    <t>Oncology Pediatric Critical Care</t>
+  </si>
+  <si>
+    <t>1119-7</t>
+  </si>
+  <si>
+    <t>Pediatric Gastrointestinal Clinic</t>
+  </si>
+  <si>
+    <t>1217-9</t>
+  </si>
+  <si>
+    <t>Rehabilitation Ward (within freestanding Inpatient Rehabilitation Facility)</t>
+  </si>
+  <si>
+    <t>1200-5</t>
+  </si>
+  <si>
+    <t>Hematology-Oncology Clinic</t>
+  </si>
+  <si>
+    <t>1152-8</t>
+  </si>
+  <si>
+    <t>Occupational Therapy Clinic</t>
+  </si>
+  <si>
+    <t>1053-8</t>
+  </si>
+  <si>
+    <t>Ear, Nose, Throat Ward</t>
+  </si>
+  <si>
+    <t>1262-1</t>
+  </si>
+  <si>
+    <t>Home Hemodialysis</t>
+  </si>
+  <si>
+    <t>1020-7</t>
+  </si>
+  <si>
+    <t>Sleep Study Unit</t>
+  </si>
+  <si>
+    <t>1143-7</t>
+  </si>
+  <si>
+    <t>Surgical Services Clinic</t>
+  </si>
+  <si>
+    <t>1012-4</t>
+  </si>
+  <si>
+    <t>Hematology Laboratory</t>
+  </si>
+  <si>
+    <t>1162-7</t>
+  </si>
+  <si>
+    <t>24-Hour Observation Area</t>
+  </si>
+  <si>
+    <t>1158-5</t>
+  </si>
+  <si>
+    <t>Speech Therapy Clinic</t>
+  </si>
+  <si>
+    <t>1097-5</t>
+  </si>
+  <si>
+    <t>Post-Anesthesia Care Unit/Recovery Room</t>
+  </si>
+  <si>
+    <t>1144-5</t>
+  </si>
+  <si>
+    <t>Wound Center</t>
+  </si>
+  <si>
+    <t>1224-5</t>
+  </si>
+  <si>
+    <t>Oncology Surgical Critical Care</t>
+  </si>
+  <si>
+    <t>1271-6</t>
+  </si>
+  <si>
+    <t>Onsite Overflow Ward</t>
+  </si>
+  <si>
+    <t>1064-5</t>
+  </si>
+  <si>
+    <t>Ophthalmology Ward</t>
+  </si>
+  <si>
+    <t>1181-7</t>
+  </si>
+  <si>
+    <t>Physical Plant Operations Center</t>
+  </si>
+  <si>
+    <t>1269-0</t>
+  </si>
+  <si>
+    <t>Neonatal Critical Care (Level IV)</t>
+  </si>
+  <si>
+    <t>1146-0</t>
+  </si>
+  <si>
+    <t>Pediatric Behavioral Health Clinic</t>
+  </si>
+  <si>
+    <t>1052-0</t>
+  </si>
+  <si>
+    <t>Burn Ward</t>
+  </si>
+  <si>
+    <t>1251-8</t>
+  </si>
+  <si>
+    <t>Facility-wide Outpatient (FacWIDEOut)</t>
+  </si>
+  <si>
+    <t>1265-8</t>
+  </si>
+  <si>
+    <t>Inpatient Psychiatric Facility Unit(s)</t>
+  </si>
+  <si>
+    <t>1041-3</t>
+  </si>
+  <si>
+    <t>Special Care Nursery (Level II)</t>
+  </si>
+  <si>
+    <t>1149-4</t>
+  </si>
+  <si>
+    <t>Ostomy Clinic</t>
+  </si>
+  <si>
+    <t>1099-1</t>
+  </si>
+  <si>
+    <t>Adult Step Down Unit</t>
+  </si>
+  <si>
+    <t>1186-6</t>
+  </si>
+  <si>
+    <t>Central Sterile Supply</t>
+  </si>
+  <si>
+    <t>1070-2</t>
+  </si>
+  <si>
+    <t>Rehabilitation Ward (within Hospital)</t>
+  </si>
+  <si>
+    <t>1013-2</t>
+  </si>
+  <si>
+    <t>Histology-Surgical Pathology Laboratory</t>
+  </si>
+  <si>
+    <t>1153-6</t>
+  </si>
+  <si>
+    <t>Outpatient Hemodialysis Clinic</t>
+  </si>
+  <si>
+    <t>1180-9</t>
+  </si>
+  <si>
+    <t>Public Area in Facility</t>
+  </si>
+  <si>
+    <t>1057-9</t>
+  </si>
+  <si>
+    <t>Gynecology Ward</t>
+  </si>
+  <si>
+    <t>1209-6</t>
+  </si>
+  <si>
+    <t>Treatment Room</t>
+  </si>
+  <si>
+    <t>1130-4</t>
+  </si>
+  <si>
+    <t>Pediatric Dental Clinic</t>
+  </si>
+  <si>
+    <t>1092-6</t>
+  </si>
+  <si>
+    <t>Solid Organ Transplant Specialty Care Area</t>
+  </si>
+  <si>
+    <t>1043-9</t>
+  </si>
+  <si>
+    <t>Pediatric Surgical Cardiothoracic Critical Care</t>
+  </si>
+  <si>
+    <t>1073-6</t>
+  </si>
+  <si>
+    <t>Vascular Surgery Ward</t>
+  </si>
+  <si>
+    <t>1155-1</t>
+  </si>
+  <si>
+    <t>Rehabilitation Clinic</t>
+  </si>
+  <si>
+    <t>1174-2</t>
+  </si>
+  <si>
+    <t>Mobile Emergency Services/EMS</t>
+  </si>
+  <si>
+    <t>1270-8</t>
+  </si>
+  <si>
+    <t>Chemical Dependency Ward</t>
+  </si>
+  <si>
+    <t>1218-7</t>
+  </si>
+  <si>
+    <t>Pediatric Rehabilitation Ward (within freestanding Inpatient Rehabilitation Facility)</t>
+  </si>
+  <si>
+    <t>1027-2</t>
+  </si>
+  <si>
+    <t>Medical Critical Care</t>
+  </si>
+  <si>
+    <t>1157-7</t>
+  </si>
+  <si>
+    <t>Pulmonary Clinic</t>
+  </si>
+  <si>
+    <t>1112-2</t>
+  </si>
+  <si>
+    <t>Cardiac Rehabilitation Center</t>
+  </si>
+  <si>
+    <t>1232-8</t>
+  </si>
+  <si>
+    <t>Oncology General Hematology-Oncology Ward</t>
+  </si>
+  <si>
+    <t>1060-3</t>
+  </si>
+  <si>
+    <t>Medical Ward</t>
+  </si>
+  <si>
+    <t>1028-0</t>
+  </si>
+  <si>
+    <t>Medical Cardiac Critical Care</t>
+  </si>
+  <si>
+    <t>1084-3</t>
+  </si>
+  <si>
+    <t>Pediatric Orthopedic Ward</t>
+  </si>
+  <si>
+    <t>1100-7</t>
+  </si>
+  <si>
+    <t>Pediatric Step Down Unit</t>
+  </si>
+  <si>
+    <t>1264-1</t>
+  </si>
+  <si>
+    <t>Inpatient Rehabilitation Facility Unit(s)</t>
+  </si>
+  <si>
+    <t>1231-0</t>
+  </si>
+  <si>
+    <t>Oncology Hematopoietic Stem Cell Transplant Ward</t>
+  </si>
+  <si>
+    <t>1206-2</t>
+  </si>
+  <si>
+    <t>Float</t>
+  </si>
+  <si>
+    <t>1030-6</t>
+  </si>
+  <si>
+    <t>Surgical Critical Care</t>
+  </si>
+  <si>
+    <t>1123-9</t>
+  </si>
+  <si>
+    <t>Neurology Clinic</t>
+  </si>
+  <si>
+    <t>1235-1</t>
+  </si>
+  <si>
+    <t>Oncology Pediatric General Hematology/Oncology Ward</t>
+  </si>
+  <si>
+    <t>1121-3</t>
+  </si>
+  <si>
+    <t>Gynecology Clinic</t>
+  </si>
+  <si>
+    <t>1047-0</t>
+  </si>
+  <si>
+    <t>Pediatric Respiratory Critical Care</t>
+  </si>
+  <si>
+    <t>1015-7</t>
+  </si>
+  <si>
+    <t>Serology Laboratory</t>
+  </si>
+  <si>
+    <t>1068-6</t>
+  </si>
+  <si>
+    <t>Postpartum Ward</t>
+  </si>
+  <si>
+    <t>1049-6</t>
+  </si>
+  <si>
+    <t>Pediatric Trauma Critical Care</t>
+  </si>
+  <si>
+    <t>1176-7</t>
+  </si>
+  <si>
+    <t>Mobile Blood Collection Center</t>
+  </si>
+  <si>
+    <t>1242-7</t>
+  </si>
+  <si>
+    <t>Outpatient Operating Room/Suite (Attached)</t>
+  </si>
+  <si>
+    <t>1170-0</t>
+  </si>
+  <si>
+    <t>School or Prison Infirmary</t>
+  </si>
+  <si>
+    <t>1072-8</t>
+  </si>
+  <si>
+    <t>Surgical Ward</t>
+  </si>
+  <si>
+    <t>1188-2</t>
+  </si>
+  <si>
+    <t>Facility Grounds</t>
+  </si>
+  <si>
+    <t>1093-4</t>
+  </si>
+  <si>
+    <t>Pediatric Solid Organ Transplant Specialty Care Area</t>
+  </si>
+  <si>
+    <t>1225-2</t>
+  </si>
+  <si>
+    <t>Oncology Medical-Surgical Critical Care</t>
+  </si>
+  <si>
+    <t>1257-5</t>
+  </si>
+  <si>
+    <t>Long Term Care Facility Skilled Nursing-Short Term Rehabilitation Unit</t>
+  </si>
+  <si>
+    <t>1228-6</t>
+  </si>
+  <si>
+    <t>Oncology Lymphoma Ward</t>
+  </si>
+  <si>
+    <t>1034-8</t>
+  </si>
+  <si>
+    <t>Prenatal Critical Care</t>
+  </si>
+  <si>
+    <t>1048-8</t>
+  </si>
+  <si>
+    <t>Pediatric Surgical Critical Care</t>
+  </si>
+  <si>
+    <t>1230-2</t>
+  </si>
+  <si>
+    <t>Oncology Solid Tumor Ward</t>
+  </si>
+  <si>
+    <t>1244-3</t>
+  </si>
+  <si>
+    <t>Outpatient Operating Room/Suite (Detached)</t>
+  </si>
+  <si>
+    <t>1063-7</t>
+  </si>
+  <si>
+    <t>Neurosurgical Ward</t>
+  </si>
+  <si>
+    <t>1208-8</t>
+  </si>
+  <si>
+    <t>Telemetry Ward</t>
+  </si>
+  <si>
+    <t>1106-4</t>
+  </si>
+  <si>
+    <t>Assisted Living Area</t>
+  </si>
+  <si>
+    <t>1120-5</t>
+  </si>
+  <si>
+    <t>Medical Clinic</t>
+  </si>
+  <si>
+    <t>1109-8</t>
+  </si>
+  <si>
+    <t>Pediatric Emergency Department</t>
+  </si>
+  <si>
+    <t>1076-9</t>
+  </si>
+  <si>
+    <t>Pediatric Medical Ward</t>
+  </si>
+  <si>
+    <t>1056-1</t>
+  </si>
+  <si>
+    <t>Gerontology Ward</t>
+  </si>
+  <si>
+    <t>1211-2</t>
+  </si>
+  <si>
+    <t>Pediatric Mixed Acuity Unit</t>
+  </si>
+  <si>
+    <t>1254-2</t>
+  </si>
+  <si>
+    <t>Long Term Care Facility Inpatient Hospice Unit</t>
+  </si>
+  <si>
+    <t>1137-9</t>
+  </si>
+  <si>
+    <t>Pediatric Nephrology Clinic</t>
+  </si>
+  <si>
+    <t>1148-6</t>
+  </si>
+  <si>
+    <t>Continence Clinic</t>
+  </si>
+  <si>
+    <t>1140-3</t>
+  </si>
+  <si>
+    <t>Podiatry Clinic</t>
+  </si>
+  <si>
+    <t>1124-7</t>
+  </si>
+  <si>
+    <t>Ophthalmology Clinic</t>
+  </si>
+  <si>
+    <t>1260-9</t>
+  </si>
+  <si>
+    <t>Long Term Care Facility Bariatric Unit</t>
+  </si>
+  <si>
+    <t>1184-1</t>
+  </si>
+  <si>
+    <t>Administrative Areas</t>
+  </si>
+  <si>
+    <t>1014-0</t>
+  </si>
+  <si>
+    <t>Microbiology Laboratory</t>
+  </si>
+  <si>
+    <t>1010-8</t>
+  </si>
+  <si>
+    <t>General Laboratory</t>
+  </si>
+  <si>
+    <t>1229-4</t>
+  </si>
+  <si>
+    <t>Oncology Leukemia-Lymphoma Ward</t>
+  </si>
+  <si>
+    <t>1236-9</t>
+  </si>
+  <si>
+    <t>Oncology Mixed Acuity Unit (all ages)</t>
+  </si>
+  <si>
+    <t>1202-1</t>
+  </si>
+  <si>
+    <t>Physical Therapy Clinic</t>
+  </si>
+  <si>
+    <t>1234-4</t>
+  </si>
+  <si>
+    <t>Oncology Pediatric Hematopoietic Stem Cell Transplant Ward</t>
+  </si>
+  <si>
+    <t>1136-1</t>
+  </si>
+  <si>
+    <t>Pediatric Hematology-Oncology Clinic</t>
+  </si>
+  <si>
+    <t>Code System</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <t>http://www.ama-assn.org/go/cpt</t>
+  </si>
+  <si>
+    <t>99213</t>
+  </si>
+  <si>
+    <t>Office or other outpatient visit for the evaluation and management of an established patient</t>
+  </si>
+  <si>
+    <t>99283</t>
+  </si>
+  <si>
+    <t>Emergency department visit</t>
+  </si>
+  <si>
+    <t>http://snomed.info/sct</t>
+  </si>
+  <si>
+    <t>183452005</t>
+  </si>
+  <si>
+    <t>Emergency hospital admission</t>
+  </si>
+  <si>
+    <t>32485007</t>
+  </si>
+  <si>
+    <t>Hospital admission</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -336,6 +1727,19 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF5B6472"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -354,10 +1758,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -379,8 +1784,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -693,10 +2106,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24" style="4" customWidth="1"/>
+    <col min="1" max="1" width="32.7109375" style="4" customWidth="1"/>
     <col min="2" max="2" width="50" style="4" customWidth="1"/>
     <col min="3" max="3" width="50.28515625" style="4" customWidth="1"/>
     <col min="4" max="4" width="39.85546875" customWidth="1"/>
@@ -742,6 +2155,7 @@
       <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
+      <c r="C6" s="11"/>
       <c r="D6" t="s">
         <v>10</v>
       </c>
@@ -878,116 +2292,98 @@
       <c r="B17" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" t="s">
         <v>39</v>
-      </c>
-      <c r="E17" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="D18" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="E18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="D19" t="s">
         <v>10</v>
       </c>
       <c r="E19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
       </c>
       <c r="E20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="D21" t="s">
         <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
       </c>
       <c r="E22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="C23" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="D23" t="s">
         <v>17</v>
       </c>
       <c r="E23" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1041,9 +2437,6 @@
       </c>
       <c r="B29" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="E29" t="s">
         <v>66</v>
@@ -1103,10 +2496,10 @@
         <v>75</v>
       </c>
       <c r="B40" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>6</v>
@@ -1117,14 +2510,17 @@
     </row>
     <row r="41" spans="1:5">
       <c r="D41" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E41" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15.75">
       <c r="A43" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D43" s="9" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1146,12 +2542,16 @@
       </c>
     </row>
     <row r="45" spans="1:5">
+      <c r="A45" s="12"/>
       <c r="E45" s="3" t="s">
         <v>85</v>
       </c>
     </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="13"/>
+    </row>
   </sheetData>
-  <dataValidations count="11">
+  <dataValidations count="12">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Max Concurrent Requests" error="Enter a whole number between 1-8" sqref="C7" xr:uid="{B2397A65-92DA-4B4E-847E-30C08B2981BC}">
       <formula1>1</formula1>
       <formula2>8</formula2>
@@ -1173,11 +2573,9 @@
       <formula2>59</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Selection" error="Please select a value only from the drop-down list provided." sqref="C28" xr:uid="{B428FB03-7507-4137-9C43-A6BB309B3265}">
-      <formula1>"Custom Fhir Path, Location Types, Managing Organizations"</formula1>
+      <formula1>"location-type, managing-org, custom-fhir-path"</formula1>
     </dataValidation>
-    <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid URL" error="Please enter a valid URL starting with http:// or https:// (e.g., https://FHIR-HOSTNAME/fhir). Spaces are not allowed." sqref="C6" xr:uid="{93AF45BC-5F5C-4D98-A709-B4493138F738}">
-      <formula1>AND(LEN(TRIM($F:$F))&gt;10,OR(LEFT(LOWER(TRIM($F:$F)),7)="http://",LEFT(LOWER(TRIM($F:$F)),8)="https://"),ISERROR(FIND(" ",$F:$F)))</formula1>
-    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6" xr:uid="{93AF45BC-5F5C-4D98-A709-B4493138F738}"/>
     <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Error" error="Enter a valid time between 00:00 and 23:59." sqref="C9" xr:uid="{16D707C9-F60B-4ED1-AFDE-8B63E55BA524}">
       <formula1>0</formula1>
       <formula2>0.999988425925926</formula2>
@@ -1194,7 +2592,1903 @@
       <formula1>0</formula1>
       <formula2>59</formula2>
     </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid port" error="Enter port value in range 1 to 65535" sqref="C20" xr:uid="{A8DEC7DD-303E-40F8-BD05-C1ACE57067D9}">
+      <formula1>1</formula1>
+      <formula2>65535</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B226"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="56.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B11" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>112</v>
+      </c>
+      <c r="B15" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>114</v>
+      </c>
+      <c r="B16" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>136</v>
+      </c>
+      <c r="B27" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>138</v>
+      </c>
+      <c r="B28" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>142</v>
+      </c>
+      <c r="B30" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>144</v>
+      </c>
+      <c r="B31" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>146</v>
+      </c>
+      <c r="B32" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>148</v>
+      </c>
+      <c r="B33" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>150</v>
+      </c>
+      <c r="B34" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>152</v>
+      </c>
+      <c r="B35" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>154</v>
+      </c>
+      <c r="B36" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>156</v>
+      </c>
+      <c r="B37" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
+        <v>158</v>
+      </c>
+      <c r="B38" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
+        <v>160</v>
+      </c>
+      <c r="B39" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>162</v>
+      </c>
+      <c r="B40" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
+        <v>164</v>
+      </c>
+      <c r="B41" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>166</v>
+      </c>
+      <c r="B42" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
+        <v>168</v>
+      </c>
+      <c r="B43" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>170</v>
+      </c>
+      <c r="B44" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>172</v>
+      </c>
+      <c r="B45" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>174</v>
+      </c>
+      <c r="B46" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
+        <v>176</v>
+      </c>
+      <c r="B47" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
+        <v>178</v>
+      </c>
+      <c r="B48" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>180</v>
+      </c>
+      <c r="B49" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>182</v>
+      </c>
+      <c r="B50" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>184</v>
+      </c>
+      <c r="B51" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
+        <v>186</v>
+      </c>
+      <c r="B52" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>188</v>
+      </c>
+      <c r="B53" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>190</v>
+      </c>
+      <c r="B54" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
+        <v>192</v>
+      </c>
+      <c r="B55" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
+        <v>194</v>
+      </c>
+      <c r="B56" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
+        <v>196</v>
+      </c>
+      <c r="B57" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
+        <v>198</v>
+      </c>
+      <c r="B58" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
+        <v>200</v>
+      </c>
+      <c r="B59" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
+        <v>202</v>
+      </c>
+      <c r="B60" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>204</v>
+      </c>
+      <c r="B61" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" t="s">
+        <v>206</v>
+      </c>
+      <c r="B62" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" t="s">
+        <v>208</v>
+      </c>
+      <c r="B63" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>210</v>
+      </c>
+      <c r="B64" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
+        <v>212</v>
+      </c>
+      <c r="B65" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" t="s">
+        <v>214</v>
+      </c>
+      <c r="B66" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" t="s">
+        <v>216</v>
+      </c>
+      <c r="B67" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
+        <v>218</v>
+      </c>
+      <c r="B68" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
+        <v>220</v>
+      </c>
+      <c r="B69" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
+        <v>222</v>
+      </c>
+      <c r="B70" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" t="s">
+        <v>224</v>
+      </c>
+      <c r="B71" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
+        <v>226</v>
+      </c>
+      <c r="B72" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
+        <v>228</v>
+      </c>
+      <c r="B73" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
+        <v>230</v>
+      </c>
+      <c r="B74" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
+        <v>232</v>
+      </c>
+      <c r="B75" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" t="s">
+        <v>234</v>
+      </c>
+      <c r="B76" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" t="s">
+        <v>236</v>
+      </c>
+      <c r="B77" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
+        <v>238</v>
+      </c>
+      <c r="B78" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
+        <v>240</v>
+      </c>
+      <c r="B79" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
+        <v>242</v>
+      </c>
+      <c r="B80" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>244</v>
+      </c>
+      <c r="B81" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>246</v>
+      </c>
+      <c r="B82" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" t="s">
+        <v>248</v>
+      </c>
+      <c r="B83" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" t="s">
+        <v>250</v>
+      </c>
+      <c r="B84" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
+        <v>252</v>
+      </c>
+      <c r="B85" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
+        <v>254</v>
+      </c>
+      <c r="B86" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" t="s">
+        <v>256</v>
+      </c>
+      <c r="B87" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" t="s">
+        <v>258</v>
+      </c>
+      <c r="B88" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
+        <v>260</v>
+      </c>
+      <c r="B89" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
+        <v>262</v>
+      </c>
+      <c r="B90" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>264</v>
+      </c>
+      <c r="B91" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>266</v>
+      </c>
+      <c r="B92" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>268</v>
+      </c>
+      <c r="B93" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
+        <v>270</v>
+      </c>
+      <c r="B94" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>272</v>
+      </c>
+      <c r="B95" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>274</v>
+      </c>
+      <c r="B96" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
+        <v>276</v>
+      </c>
+      <c r="B97" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" t="s">
+        <v>278</v>
+      </c>
+      <c r="B98" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
+        <v>280</v>
+      </c>
+      <c r="B99" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
+        <v>282</v>
+      </c>
+      <c r="B100" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" t="s">
+        <v>284</v>
+      </c>
+      <c r="B101" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" t="s">
+        <v>286</v>
+      </c>
+      <c r="B102" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" t="s">
+        <v>288</v>
+      </c>
+      <c r="B103" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" t="s">
+        <v>290</v>
+      </c>
+      <c r="B104" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" t="s">
+        <v>292</v>
+      </c>
+      <c r="B105" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" t="s">
+        <v>294</v>
+      </c>
+      <c r="B106" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" t="s">
+        <v>296</v>
+      </c>
+      <c r="B107" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" t="s">
+        <v>298</v>
+      </c>
+      <c r="B108" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" t="s">
+        <v>300</v>
+      </c>
+      <c r="B109" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" t="s">
+        <v>302</v>
+      </c>
+      <c r="B110" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" t="s">
+        <v>304</v>
+      </c>
+      <c r="B111" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" t="s">
+        <v>306</v>
+      </c>
+      <c r="B112" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" t="s">
+        <v>308</v>
+      </c>
+      <c r="B113" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" t="s">
+        <v>310</v>
+      </c>
+      <c r="B114" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" t="s">
+        <v>312</v>
+      </c>
+      <c r="B115" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" t="s">
+        <v>314</v>
+      </c>
+      <c r="B116" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" t="s">
+        <v>316</v>
+      </c>
+      <c r="B117" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" t="s">
+        <v>318</v>
+      </c>
+      <c r="B118" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" t="s">
+        <v>320</v>
+      </c>
+      <c r="B119" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" t="s">
+        <v>322</v>
+      </c>
+      <c r="B120" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" t="s">
+        <v>324</v>
+      </c>
+      <c r="B121" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" t="s">
+        <v>326</v>
+      </c>
+      <c r="B122" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" t="s">
+        <v>328</v>
+      </c>
+      <c r="B123" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" t="s">
+        <v>330</v>
+      </c>
+      <c r="B124" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" t="s">
+        <v>332</v>
+      </c>
+      <c r="B125" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" t="s">
+        <v>334</v>
+      </c>
+      <c r="B126" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" t="s">
+        <v>336</v>
+      </c>
+      <c r="B127" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" t="s">
+        <v>338</v>
+      </c>
+      <c r="B128" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" t="s">
+        <v>340</v>
+      </c>
+      <c r="B129" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" t="s">
+        <v>342</v>
+      </c>
+      <c r="B130" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" t="s">
+        <v>344</v>
+      </c>
+      <c r="B131" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" t="s">
+        <v>346</v>
+      </c>
+      <c r="B132" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" t="s">
+        <v>348</v>
+      </c>
+      <c r="B133" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" t="s">
+        <v>350</v>
+      </c>
+      <c r="B134" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" t="s">
+        <v>352</v>
+      </c>
+      <c r="B135" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" t="s">
+        <v>354</v>
+      </c>
+      <c r="B136" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" t="s">
+        <v>356</v>
+      </c>
+      <c r="B137" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" t="s">
+        <v>358</v>
+      </c>
+      <c r="B138" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" t="s">
+        <v>360</v>
+      </c>
+      <c r="B139" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" t="s">
+        <v>362</v>
+      </c>
+      <c r="B140" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" t="s">
+        <v>364</v>
+      </c>
+      <c r="B141" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" t="s">
+        <v>366</v>
+      </c>
+      <c r="B142" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" t="s">
+        <v>368</v>
+      </c>
+      <c r="B143" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" t="s">
+        <v>370</v>
+      </c>
+      <c r="B144" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" t="s">
+        <v>372</v>
+      </c>
+      <c r="B145" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" t="s">
+        <v>374</v>
+      </c>
+      <c r="B146" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" t="s">
+        <v>376</v>
+      </c>
+      <c r="B147" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" t="s">
+        <v>378</v>
+      </c>
+      <c r="B148" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" t="s">
+        <v>380</v>
+      </c>
+      <c r="B149" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" t="s">
+        <v>382</v>
+      </c>
+      <c r="B150" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" t="s">
+        <v>384</v>
+      </c>
+      <c r="B151" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" t="s">
+        <v>386</v>
+      </c>
+      <c r="B152" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" t="s">
+        <v>388</v>
+      </c>
+      <c r="B153" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" t="s">
+        <v>390</v>
+      </c>
+      <c r="B154" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" t="s">
+        <v>392</v>
+      </c>
+      <c r="B155" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" t="s">
+        <v>394</v>
+      </c>
+      <c r="B156" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" t="s">
+        <v>396</v>
+      </c>
+      <c r="B157" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" t="s">
+        <v>398</v>
+      </c>
+      <c r="B158" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" t="s">
+        <v>400</v>
+      </c>
+      <c r="B159" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" t="s">
+        <v>402</v>
+      </c>
+      <c r="B160" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" t="s">
+        <v>404</v>
+      </c>
+      <c r="B161" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" t="s">
+        <v>406</v>
+      </c>
+      <c r="B162" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" t="s">
+        <v>408</v>
+      </c>
+      <c r="B163" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" t="s">
+        <v>410</v>
+      </c>
+      <c r="B164" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" t="s">
+        <v>412</v>
+      </c>
+      <c r="B165" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" t="s">
+        <v>414</v>
+      </c>
+      <c r="B166" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" t="s">
+        <v>416</v>
+      </c>
+      <c r="B167" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" t="s">
+        <v>418</v>
+      </c>
+      <c r="B168" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" t="s">
+        <v>420</v>
+      </c>
+      <c r="B169" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" t="s">
+        <v>422</v>
+      </c>
+      <c r="B170" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2">
+      <c r="A171" t="s">
+        <v>424</v>
+      </c>
+      <c r="B171" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2">
+      <c r="A172" t="s">
+        <v>426</v>
+      </c>
+      <c r="B172" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2">
+      <c r="A173" t="s">
+        <v>428</v>
+      </c>
+      <c r="B173" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2">
+      <c r="A174" t="s">
+        <v>430</v>
+      </c>
+      <c r="B174" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2">
+      <c r="A175" t="s">
+        <v>432</v>
+      </c>
+      <c r="B175" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
+      <c r="A176" t="s">
+        <v>434</v>
+      </c>
+      <c r="B176" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
+      <c r="A177" t="s">
+        <v>436</v>
+      </c>
+      <c r="B177" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
+      <c r="A178" t="s">
+        <v>438</v>
+      </c>
+      <c r="B178" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
+      <c r="A179" t="s">
+        <v>440</v>
+      </c>
+      <c r="B179" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2">
+      <c r="A180" t="s">
+        <v>442</v>
+      </c>
+      <c r="B180" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2">
+      <c r="A181" t="s">
+        <v>444</v>
+      </c>
+      <c r="B181" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
+      <c r="A182" t="s">
+        <v>446</v>
+      </c>
+      <c r="B182" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
+      <c r="A183" t="s">
+        <v>448</v>
+      </c>
+      <c r="B183" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
+      <c r="A184" t="s">
+        <v>450</v>
+      </c>
+      <c r="B184" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
+      <c r="A185" t="s">
+        <v>452</v>
+      </c>
+      <c r="B185" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2">
+      <c r="A186" t="s">
+        <v>454</v>
+      </c>
+      <c r="B186" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2">
+      <c r="A187" t="s">
+        <v>456</v>
+      </c>
+      <c r="B187" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" t="s">
+        <v>458</v>
+      </c>
+      <c r="B188" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" t="s">
+        <v>460</v>
+      </c>
+      <c r="B189" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" t="s">
+        <v>462</v>
+      </c>
+      <c r="B190" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" t="s">
+        <v>464</v>
+      </c>
+      <c r="B191" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2">
+      <c r="A192" t="s">
+        <v>466</v>
+      </c>
+      <c r="B192" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" t="s">
+        <v>468</v>
+      </c>
+      <c r="B193" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2">
+      <c r="A194" t="s">
+        <v>470</v>
+      </c>
+      <c r="B194" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2">
+      <c r="A195" t="s">
+        <v>472</v>
+      </c>
+      <c r="B195" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2">
+      <c r="A196" t="s">
+        <v>474</v>
+      </c>
+      <c r="B196" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2">
+      <c r="A197" t="s">
+        <v>476</v>
+      </c>
+      <c r="B197" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2">
+      <c r="A198" t="s">
+        <v>478</v>
+      </c>
+      <c r="B198" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2">
+      <c r="A199" t="s">
+        <v>480</v>
+      </c>
+      <c r="B199" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2">
+      <c r="A200" t="s">
+        <v>482</v>
+      </c>
+      <c r="B200" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2">
+      <c r="A201" t="s">
+        <v>484</v>
+      </c>
+      <c r="B201" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2">
+      <c r="A202" t="s">
+        <v>486</v>
+      </c>
+      <c r="B202" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2">
+      <c r="A203" t="s">
+        <v>488</v>
+      </c>
+      <c r="B203" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2">
+      <c r="A204" t="s">
+        <v>490</v>
+      </c>
+      <c r="B204" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2">
+      <c r="A205" t="s">
+        <v>492</v>
+      </c>
+      <c r="B205" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2">
+      <c r="A206" t="s">
+        <v>494</v>
+      </c>
+      <c r="B206" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2">
+      <c r="A207" t="s">
+        <v>496</v>
+      </c>
+      <c r="B207" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2">
+      <c r="A208" t="s">
+        <v>498</v>
+      </c>
+      <c r="B208" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
+      <c r="A209" t="s">
+        <v>500</v>
+      </c>
+      <c r="B209" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
+      <c r="A210" t="s">
+        <v>502</v>
+      </c>
+      <c r="B210" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
+      <c r="A211" t="s">
+        <v>504</v>
+      </c>
+      <c r="B211" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
+      <c r="A212" t="s">
+        <v>506</v>
+      </c>
+      <c r="B212" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
+      <c r="A213" t="s">
+        <v>508</v>
+      </c>
+      <c r="B213" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" t="s">
+        <v>510</v>
+      </c>
+      <c r="B214" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" t="s">
+        <v>512</v>
+      </c>
+      <c r="B215" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" t="s">
+        <v>514</v>
+      </c>
+      <c r="B216" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" t="s">
+        <v>516</v>
+      </c>
+      <c r="B217" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" t="s">
+        <v>518</v>
+      </c>
+      <c r="B218" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" t="s">
+        <v>520</v>
+      </c>
+      <c r="B219" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" t="s">
+        <v>522</v>
+      </c>
+      <c r="B220" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" t="s">
+        <v>524</v>
+      </c>
+      <c r="B221" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" t="s">
+        <v>526</v>
+      </c>
+      <c r="B222" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" t="s">
+        <v>528</v>
+      </c>
+      <c r="B223" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" t="s">
+        <v>530</v>
+      </c>
+      <c r="B224" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" t="s">
+        <v>532</v>
+      </c>
+      <c r="B225" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2">
+      <c r="A226" t="s">
+        <v>534</v>
+      </c>
+      <c r="B226" t="s">
+        <v>535</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="83" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="9" t="s">
+        <v>536</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>539</v>
+      </c>
+      <c r="B2" t="s">
+        <v>540</v>
+      </c>
+      <c r="C2" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>539</v>
+      </c>
+      <c r="B3" t="s">
+        <v>542</v>
+      </c>
+      <c r="C3" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>544</v>
+      </c>
+      <c r="B4" t="s">
+        <v>545</v>
+      </c>
+      <c r="C4" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>544</v>
+      </c>
+      <c r="B5" t="s">
+        <v>547</v>
+      </c>
+      <c r="C5" t="s">
+        <v>548</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+</worksheet>
 </file>
</xml_diff>